<commit_message>
Fix NDVI period naming and strengthen reproducibility checks
</commit_message>
<xml_diff>
--- a/results/diagnostics/20_FINAL_DIAGNOSTICS.xlsx
+++ b/results/diagnostics/20_FINAL_DIAGNOSTICS.xlsx
@@ -6,20 +6,23 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Descriptive" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Within_variation" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Livestock" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Within_correlations" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Descriptive statistics" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Raw correlations" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Two-way correlations" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Within variation" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t xml:space="preserve">Variable</t>
   </si>
   <si>
+    <t xml:space="preserve">N</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mean</t>
   </si>
   <si>
@@ -32,12 +35,12 @@
     <t xml:space="preserve">Max</t>
   </si>
   <si>
+    <t xml:space="preserve">RRUI</t>
+  </si>
+  <si>
     <t xml:space="preserve">NDVI</t>
   </si>
   <si>
-    <t xml:space="preserve">RRUI</t>
-  </si>
-  <si>
     <t xml:space="preserve">precip_mm</t>
   </si>
   <si>
@@ -50,12 +53,15 @@
     <t xml:space="preserve">ADM2_PCODE</t>
   </si>
   <si>
-    <t xml:space="preserve">N</t>
+    <t xml:space="preserve">ADM2_EN</t>
   </si>
   <si>
     <t xml:space="preserve">RRUI_SD</t>
   </si>
   <si>
+    <t xml:space="preserve">NDVI_SD</t>
+  </si>
+  <si>
     <t xml:space="preserve">Precip_SD</t>
   </si>
   <si>
@@ -68,49 +74,31 @@
     <t xml:space="preserve">KAZ020001</t>
   </si>
   <si>
+    <t xml:space="preserve">Akzhaik District</t>
+  </si>
+  <si>
     <t xml:space="preserve">KAZ020002</t>
   </si>
   <si>
+    <t xml:space="preserve">Bokey Orda District</t>
+  </si>
+  <si>
     <t xml:space="preserve">KAZ020005</t>
   </si>
   <si>
+    <t xml:space="preserve">Kaztal District</t>
+  </si>
+  <si>
     <t xml:space="preserve">KAZ020012</t>
   </si>
   <si>
+    <t xml:space="preserve">Zhanakala District</t>
+  </si>
+  <si>
     <t xml:space="preserve">KAZ020013</t>
   </si>
   <si>
-    <t xml:space="preserve">ADM2_EN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Akzhaik District</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bokey Orda District</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kaztal District</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zhanakala District</t>
-  </si>
-  <si>
     <t xml:space="preserve">Zhanybek District</t>
-  </si>
-  <si>
-    <t xml:space="preserve"/>
-  </si>
-  <si>
-    <t xml:space="preserve">RRUI_within</t>
-  </si>
-  <si>
-    <t xml:space="preserve">precip_within</t>
-  </si>
-  <si>
-    <t xml:space="preserve">temp_within</t>
-  </si>
-  <si>
-    <t xml:space="preserve">livestock_within</t>
   </si>
 </sst>
 </file>
@@ -455,89 +443,107 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.2950090204309</v>
+        <v>65</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0448147441932345</v>
+        <v>0.2</v>
       </c>
       <c r="D2" t="n">
-        <v>0.217935382884302</v>
+        <v>0.186975004575886</v>
       </c>
       <c r="E2" t="n">
-        <v>0.425417855421011</v>
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.625603921149873</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B3" t="n">
-        <v>0.2</v>
+        <v>65</v>
       </c>
       <c r="C3" t="n">
-        <v>0.186975004575886</v>
+        <v>0.2950090204309</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>0.0448147441932345</v>
       </c>
       <c r="E3" t="n">
-        <v>0.625603921149873</v>
+        <v>0.217935382884302</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.425417855421011</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B4" t="n">
+        <v>65</v>
+      </c>
+      <c r="C4" t="n">
         <v>146.873804355744</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>31.9857557595652</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>87.8063541211719</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>221.553950182883</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" t="n">
+        <v>65</v>
+      </c>
+      <c r="C5" t="n">
         <v>19.0145292167617</v>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
         <v>0.716086140178332</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>17.9012756020899</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>21.1778556470097</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6" t="n">
+        <v>65</v>
+      </c>
+      <c r="C6" t="n">
         <v>119.072624615385</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>45.1934591309062</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>37.144</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>236.3</v>
       </c>
     </row>
@@ -554,122 +560,87 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" t="s">
         <v>10</v>
-      </c>
-      <c r="B1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F1" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0314633011989358</v>
+        <v>0.365616063516761</v>
       </c>
       <c r="D2" t="n">
-        <v>29.4765863089018</v>
+        <v>-0.140542314573349</v>
       </c>
       <c r="E2" t="n">
-        <v>0.725008373099377</v>
-      </c>
-      <c r="F2" t="n">
-        <v>38.7507588060031</v>
+        <v>-0.243912696359426</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="B3" t="n">
-        <v>13</v>
+        <v>0.365616063516761</v>
       </c>
       <c r="C3" t="n">
-        <v>0.207833509904493</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>22.7274168078289</v>
+        <v>-0.284463902291939</v>
       </c>
       <c r="E3" t="n">
-        <v>0.530691286782258</v>
-      </c>
-      <c r="F3" t="n">
-        <v>24.4617277512423</v>
+        <v>-0.1925789708053</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B4" t="n">
-        <v>13</v>
+        <v>-0.140542314573349</v>
       </c>
       <c r="C4" t="n">
-        <v>0.156925072389753</v>
+        <v>-0.284463902291939</v>
       </c>
       <c r="D4" t="n">
-        <v>25.1950357700839</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>0.583417245394264</v>
-      </c>
-      <c r="F4" t="n">
-        <v>43.5849523450115</v>
+        <v>-0.0201407131616609</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="B5" t="n">
-        <v>13</v>
+        <v>-0.243912696359426</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0855133771887513</v>
+        <v>-0.1925789708053</v>
       </c>
       <c r="D5" t="n">
-        <v>23.5743262108591</v>
+        <v>-0.0201407131616609</v>
       </c>
       <c r="E5" t="n">
-        <v>0.593716553096843</v>
-      </c>
-      <c r="F5" t="n">
-        <v>25.3811219982036</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" t="n">
-        <v>13</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0.140055854518727</v>
-      </c>
-      <c r="D6" t="n">
-        <v>29.2331856617582</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.612586091968236</v>
-      </c>
-      <c r="F6" t="n">
-        <v>22.2229348319046</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -685,122 +656,87 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" t="s">
         <v>10</v>
-      </c>
-      <c r="B1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" t="s">
-        <v>22</v>
+        <v>6</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>100.9918</v>
+        <v>-0.00891641248591383</v>
       </c>
       <c r="D2" t="n">
-        <v>157.572153846154</v>
+        <v>0.0292106195330673</v>
       </c>
       <c r="E2" t="n">
-        <v>236.22</v>
-      </c>
-      <c r="F2" t="n">
-        <v>38.7507588060031</v>
+        <v>-0.257116502896031</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" t="s">
-        <v>23</v>
+        <v>8</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-0.00891641248591383</v>
       </c>
       <c r="C3" t="n">
-        <v>75.4766</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>108.577461538462</v>
+        <v>-0.435528024934217</v>
       </c>
       <c r="E3" t="n">
-        <v>158.32</v>
-      </c>
-      <c r="F3" t="n">
-        <v>24.4617277512423</v>
+        <v>0.133118667771508</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" t="s">
-        <v>24</v>
+        <v>9</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0.0292106195330673</v>
       </c>
       <c r="C4" t="n">
-        <v>86.0594</v>
+        <v>-0.435528024934217</v>
       </c>
       <c r="D4" t="n">
-        <v>150.081276923077</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>236.3</v>
-      </c>
-      <c r="F4" t="n">
-        <v>43.5849523450115</v>
+        <v>-0.0796730701805873</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" t="s">
-        <v>25</v>
+        <v>10</v>
+      </c>
+      <c r="B5" t="n">
+        <v>-0.257116502896031</v>
       </c>
       <c r="C5" t="n">
-        <v>73.5816</v>
+        <v>0.133118667771508</v>
       </c>
       <c r="D5" t="n">
-        <v>112.121246153846</v>
+        <v>-0.0796730701805873</v>
       </c>
       <c r="E5" t="n">
-        <v>156.2842</v>
-      </c>
-      <c r="F5" t="n">
-        <v>25.3811219982036</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" t="n">
-        <v>37.144</v>
-      </c>
-      <c r="D6" t="n">
-        <v>67.0109846153846</v>
-      </c>
-      <c r="E6" t="n">
-        <v>109.2</v>
-      </c>
-      <c r="F6" t="n">
-        <v>22.2229348319046</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -816,87 +752,140 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="B1" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="C1" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="D1" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E1" t="s">
-        <v>31</v>
+        <v>15</v>
+      </c>
+      <c r="F1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" t="n">
-        <v>1</v>
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.00891641248591383</v>
+        <v>0.0314633011989358</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0292106195330673</v>
+        <v>0.0441671847571708</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.257116502896031</v>
+        <v>29.4765863089018</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.725008373099377</v>
+      </c>
+      <c r="G2" t="n">
+        <v>38.7507588060031</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B3" t="n">
-        <v>-0.00891641248591383</v>
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
+        <v>21</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>0.207833509904493</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.435528024934217</v>
+        <v>0.0279510668729034</v>
       </c>
       <c r="E3" t="n">
-        <v>0.133118667771508</v>
+        <v>22.7274168078289</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.530691286782258</v>
+      </c>
+      <c r="G3" t="n">
+        <v>24.4617277512423</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.0292106195330673</v>
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
+        <v>23</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.435528024934217</v>
+        <v>0.156925072389753</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0.0378773246031385</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.0796730701805873</v>
+        <v>25.1950357700839</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.583417245394264</v>
+      </c>
+      <c r="G4" t="n">
+        <v>43.5849523450115</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B5" t="n">
-        <v>-0.257116502896031</v>
+        <v>24</v>
+      </c>
+      <c r="B5" t="s">
+        <v>25</v>
       </c>
       <c r="C5" t="n">
-        <v>0.133118667771508</v>
+        <v>0.0855133771887513</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.0796730701805873</v>
+        <v>0.0258686221509113</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>23.5743262108591</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.593716553096843</v>
+      </c>
+      <c r="G5" t="n">
+        <v>25.3811219982036</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.140055854518727</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.0460514899875677</v>
+      </c>
+      <c r="E6" t="n">
+        <v>29.2331856617582</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.612586091968236</v>
+      </c>
+      <c r="G6" t="n">
+        <v>22.2229348319046</v>
       </c>
     </row>
   </sheetData>

</xml_diff>